<commit_message>
FIX: Fixes from Copilot
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/DATE.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/DATE.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shalom/workspace/projects/IronCalc/xlsx/tests/calc_tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Downloads/sort/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BA086BD-5FB1-4F48-AA24-6CEA19F71945}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D95CEBEA-5D6D-0E4A-A173-FF6D1EAF408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" xr2:uid="{C2CB1143-6AA3-1E48-BD1F-81E601D12BF5}"/>
+    <workbookView xWindow="5580" yWindow="2300" windowWidth="27640" windowHeight="16940" activeTab="1" xr2:uid="{C2CB1143-6AA3-1E48-BD1F-81E601D12BF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Arrays" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="4">
   <si>
     <t>YEAR</t>
   </si>
@@ -620,4 +643,177 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B7FF1FD-B6A3-764B-9560-52A3182E8DB5}">
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" cm="1">
+        <f t="array" ref="E1:E5">DATE(A2:A6,1,1)</f>
+        <v>44562</v>
+      </c>
+      <c r="G1" s="1" cm="1">
+        <f t="array" ref="G1:G5">DATE(A2:A6,B2:B4,C2:C3)</f>
+        <v>44562</v>
+      </c>
+      <c r="I1" s="1" cm="1">
+        <f t="array" ref="I1:I5">DATE(A2:A6,B2:B6,C2:C6)</f>
+        <v>44562</v>
+      </c>
+      <c r="K1" s="1" cm="1">
+        <f t="array" ref="K1:K5">DATE(2027,B2:B6,1)</f>
+        <v>46388</v>
+      </c>
+      <c r="M1" s="1" cm="1">
+        <f t="array" ref="M1:M5">DATE(2027,2,C2:C6)</f>
+        <v>46419</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A2">
+        <v>2022</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>44927</v>
+      </c>
+      <c r="G2">
+        <v>45201</v>
+      </c>
+      <c r="I2">
+        <v>45201</v>
+      </c>
+      <c r="K2">
+        <v>46661</v>
+      </c>
+      <c r="M2">
+        <v>46420</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A3">
+        <v>2023</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>45292</v>
+      </c>
+      <c r="G3" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I3">
+        <v>45564</v>
+      </c>
+      <c r="K3">
+        <v>46631</v>
+      </c>
+      <c r="M3">
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <v>2024</v>
+      </c>
+      <c r="B4">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>29</v>
+      </c>
+      <c r="E4">
+        <v>45658</v>
+      </c>
+      <c r="G4" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I4">
+        <v>45841</v>
+      </c>
+      <c r="K4">
+        <v>46569</v>
+      </c>
+      <c r="M4">
+        <v>46421</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5">
+        <v>2025</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>46023</v>
+      </c>
+      <c r="G5" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I5">
+        <v>46152</v>
+      </c>
+      <c r="K5">
+        <v>46508</v>
+      </c>
+      <c r="M5">
+        <v>46428</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <v>2026</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" cm="1">
+        <f t="array" ref="A10:B11">DATE({2023,2024;2025,2026}, 1, 2)</f>
+        <v>44928</v>
+      </c>
+      <c r="B10">
+        <v>45293</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>45659</v>
+      </c>
+      <c r="B11">
+        <v>46024</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>